<commit_message>
Visible boxes on bookmark/review buttons, add .rv class, trim repeated note (build 10)
</commit_message>
<xml_diff>
--- a/IDW-Sonic-reading-order.xlsx
+++ b/IDW-Sonic-reading-order.xlsx
@@ -572,7 +572,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Also included in Sonic Origins (2022), which is not tracked separately as a compilation.</t>
+          <t>In Sonic Origins (2022).</t>
         </is>
       </c>
       <c r="L2" s="2" t="n"/>
@@ -619,7 +619,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Also included in Sonic Origins (2022), which is not tracked separately as a compilation.</t>
+          <t>In Sonic Origins (2022).</t>
         </is>
       </c>
       <c r="L3" s="2" t="n"/>
@@ -1802,7 +1802,7 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Also included in Sonic Origins (2022), which is not tracked separately as a compilation.</t>
+          <t>In Sonic Origins (2022).</t>
         </is>
       </c>
       <c r="L28" s="2" t="n"/>
@@ -5280,7 +5280,7 @@
       <c r="J102" s="2" t="inlineStr"/>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>Also included in Sonic Origins (2022), which is not tracked separately as a compilation.</t>
+          <t>In Sonic Origins (2022).</t>
         </is>
       </c>
       <c r="L102" s="2" t="n"/>
@@ -6502,7 +6502,7 @@
       <c r="J128" s="2" t="inlineStr"/>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>Also included in Sonic Origins (2022), which is not tracked separately as a compilation.</t>
+          <t>In Sonic Origins (2022).</t>
         </is>
       </c>
       <c r="L128" s="2" t="n"/>

</xml_diff>